<commit_message>
Update comparison with additional Korean literature mappings
</commit_message>
<xml_diff>
--- a/docs/data/genotype_comparison_20261027.xlsx
+++ b/docs/data/genotype_comparison_20261027.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="R2c54bc10129a415d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="Rb9d0704507c74ee4"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -750,17 +750,19 @@
         <x:v>[1] Cha Ra Mi et al. (2025). Genetic characteristics and pathogenesis of clade 2.3.4.4b H5N1 high pathogenicity avian influenza virus isolated from poultry in South Korea, 2022–2023. Virus Research. https://doi.org/10.1016/j.virusres.2025.199541</x:v>
       </x:c>
     </x:row>
-    <x:row r="24" ht="102" customHeight="1">
+    <x:row r="24" ht="162" customHeight="1">
       <x:c r="A24" s="7" t="str">
         <x:v>AS-c.3.1</x:v>
       </x:c>
       <x:c r="B24" s="7" t="str">
         <x:v>G2c-13 [1]
-Genotype 2 [2]</x:v>
+Genotype 2 [2]
+Kor24–25A [3]</x:v>
       </x:c>
       <x:c r="C24" s="7" t="str">
         <x:v>[1] Takadate Yoshihiro et al. (2026). High pathogenicity avian influenza A (H5N1) viruses isolated from poultry and wild birds in Japan during the 2024–2025 season. Microbiology Spectrum. https://doi.org/10.1128/spectrum.00293-26
-[2] Si Young-Jae et al. (2025). First detection of clade 2.3.4.4b H5N1 highly pathogenic avian influenza virus in a wild leopard cat (Prionailurus bengalensis) in South Korea. Frontiers in Veterinary Science. https://doi.org/10.3389/fvets.2025.1638067</x:v>
+[2] Si Young-Jae et al. (2025). First detection of clade 2.3.4.4b H5N1 highly pathogenic avian influenza virus in a wild leopard cat (Prionailurus bengalensis) in South Korea. Frontiers in Veterinary Science. https://doi.org/10.3389/fvets.2025.1638067
+[3] Seo Ye-Ram et al. (2026). Multiple introductions and spread of novel reassortant highly pathogenic avian influenza A (H5N1) clade 2.3.4.4b viruses via wild birds, South Korea, 2024–2025. Veterinary Research, 57, 178. https://doi.org/10.1186/s13567-026-01847-2</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="48" customHeight="1">
@@ -787,7 +789,7 @@
 [2] Cha Ra Mi et al. (2026). Emergence and Genetic Characteristics of H5N1, H5N6, and H5N3 Clade 2.3.4.4b High Pathogenicity Avian Influenza Viruses in South Korea During the 2023–2024 and 2024–2025 Winter Seasons. Transboundary and Emerging Diseases. https://doi.org/10.1155/tbed/8053623</x:v>
       </x:c>
     </x:row>
-    <x:row r="27" ht="237" customHeight="1">
+    <x:row r="27" ht="297" customHeight="1">
       <x:c r="A27" s="7" t="str">
         <x:v>AS-d.1</x:v>
       </x:c>
@@ -795,13 +797,15 @@
         <x:v>G2d-0 [1]
 I [2]
 G1 [3]
-22G0 [4]</x:v>
+22G0 [4]
+Kor24–25B [5]</x:v>
       </x:c>
       <x:c r="C27" s="7" t="str">
         <x:v>[1] Takadate Yoshihiro et al. (2024). Genetic diversity of H5N1 and H5N2 high pathogenicity avian influenza viruses isolated from poultry in Japan during the winter of 2022–2023. Virus Research. https://doi.org/10.1016/j.virusres.2024.199425
 [2] Hew Lim Yik et al. (2024). Continuous Introduction of H5 High Pathogenicity Avian Influenza Viruses in Hokkaido, Japan: Characterization of Viruses Isolated in Winter 2022–2023 and Early Winter 2023–2024. Transboundary and Emerging Diseases. https://doi.org/10.1155/2024/1199876
 [3] Cui Pengfei et al. (2022). Global dissemination of H5N1 influenza viruses bearing the clade 2.3.4.4b HA gene and biologic analysis of the ones detected in China. Emerging Microbes &amp; Infections. https://doi.org/10.1080/22221751.2022.2088407
-[4] Cha Ra Mi et al. (2025). Genetic characteristics and pathogenesis of clade 2.3.4.4b H5N1 high pathogenicity avian influenza virus isolated from poultry in South Korea, 2022–2023. Virus Research. https://doi.org/10.1016/j.virusres.2025.199541</x:v>
+[4] Cha Ra Mi et al. (2025). Genetic characteristics and pathogenesis of clade 2.3.4.4b H5N1 high pathogenicity avian influenza virus isolated from poultry in South Korea, 2022–2023. Virus Research. https://doi.org/10.1016/j.virusres.2025.199541
+[5] Seo Ye-Ram et al. (2026). Multiple introductions and spread of novel reassortant highly pathogenic avian influenza A (H5N1) clade 2.3.4.4b viruses via wild birds, South Korea, 2024–2025. Veterinary Research, 57, 178. https://doi.org/10.1186/s13567-026-01847-2</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="117" customHeight="1">
@@ -1239,10 +1243,16 @@
         <x:v>[1] Takadate Yoshihiro et al. (2026). High pathogenicity avian influenza A (H5N1) viruses isolated from poultry and wild birds in Japan during the 2024–2025 season. Microbiology Spectrum. https://doi.org/10.1128/spectrum.00293-26</x:v>
       </x:c>
     </x:row>
-    <x:row r="67" ht="33.75">
-      <x:c r="A67" s="2"/>
-      <x:c r="B67" s="2"/>
-      <x:c r="C67" s="2"/>
+    <x:row r="67" ht="57" customHeight="1">
+      <x:c r="A67" s="6" t="str">
+        <x:v>minor68</x:v>
+      </x:c>
+      <x:c r="B67" s="6" t="str">
+        <x:v>Kor24–25C [1]</x:v>
+      </x:c>
+      <x:c r="C67" s="6" t="str">
+        <x:v>[1] Seo Ye-Ram et al. (2026). Multiple introductions and spread of novel reassortant highly pathogenic avian influenza A (H5N1) clade 2.3.4.4b viruses via wild birds, South Korea, 2024–2025. Veterinary Research, 57, 178. https://doi.org/10.1186/s13567-026-01847-2</x:v>
+      </x:c>
     </x:row>
     <x:row r="68" ht="33.75">
       <x:c r="A68" s="3"/>

</xml_diff>

<commit_message>
Add missing literature correspondences to genotype comparison
</commit_message>
<xml_diff>
--- a/docs/data/genotype_comparison_20261027.xlsx
+++ b/docs/data/genotype_comparison_20261027.xlsx
@@ -2,7 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="Rb9d0704507c74ee4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="Ref5a0dba797f483e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Excluded accession" sheetId="2" r:id="Rfdd1f21d89ca4652"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -13,7 +14,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:fonts count="4">
+  <x:fonts count="6">
     <x:font>
       <x:sz val="11"/>
       <x:color theme="1"/>
@@ -40,8 +41,23 @@
       <x:name val="Malgun Gothic"/>
       <x:family val="3"/>
     </x:font>
+    <x:font>
+      <x:sz val="11"/>
+      <x:color theme="1"/>
+      <x:name val="Malgun Gothic"/>
+      <x:family val="2"/>
+      <x:scheme val="minor"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color theme="1"/>
+      <x:name val="Malgun Gothic"/>
+      <x:family val="2"/>
+      <x:scheme val="minor"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="5">
+  <x:fills count="7">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -61,6 +77,16 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FFF3F6F9"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFDCE7EF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF2CC"/>
       </x:patternFill>
     </x:fill>
   </x:fills>
@@ -98,7 +124,7 @@
       <x:alignment vertical="center"/>
     </x:xf>
   </x:cellStyleXfs>
-  <x:cellXfs count="9">
+  <x:cellXfs count="15">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <x:alignment vertical="center"/>
     </x:xf>
@@ -124,6 +150,24 @@
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -613,7 +657,7 @@
 [3] Cha Ra Mi et al. (2025). Genetic characteristics and pathogenesis of clade 2.3.4.4b H5N1 high pathogenicity avian influenza virus isolated from poultry in South Korea, 2022–2023. Virus Research. https://doi.org/10.1016/j.virusres.2025.199541</x:v>
       </x:c>
     </x:row>
-    <x:row r="14" ht="372" customHeight="1">
+    <x:row r="14" ht="409" customHeight="1">
       <x:c r="A14" s="7" t="str">
         <x:v>AS-c.2</x:v>
       </x:c>
@@ -625,7 +669,8 @@
 VI [4]
 South Korean genotype III [5]
 Kor22-23D [6]
-22G7 [7]</x:v>
+22G7 [7]
+H5N1-XII [8]</x:v>
       </x:c>
       <x:c r="C14" s="7" t="str">
         <x:v>[1] Barman Subrata et al. (2024). Reassortment of newly emergent clade 2.3.4.4b A(H5N1) highly pathogenic avian influenza A viruses in Bangladesh. Emerging Microbes &amp; Infections. https://doi.org/10.1080/22221751.2024.2432351
@@ -634,7 +679,8 @@
 [4] Hew Lim Yik et al. (2024). Continuous Introduction of H5 High Pathogenicity Avian Influenza Viruses in Hokkaido, Japan: Characterization of Viruses Isolated in Winter 2022–2023 and Early Winter 2023–2024. Transboundary and Emerging Diseases. https://doi.org/10.1155/2024/1199876
 [5] Lee Kyungmoon et al. (2024). Characterization of highly pathogenic avian influenza A (H5N1) viruses isolated from cats in South Korea, 2023. Emerging Microbes &amp; Infections. https://doi.org/10.1080/22221751.2023.2290835
 [6] Seo Ye-Ram et al. (2024). Evolution and Spread of Highly Pathogenic Avian Influenza A(H5N1) Clade 2.3.4.4b Virus in Wild Birds, South Korea, 2022–2023. Emerging Infectious Diseases. https://doi.org/10.3201/eid3002.231274
-[7] Cha Ra Mi et al. (2025). Genetic characteristics and pathogenesis of clade 2.3.4.4b H5N1 high pathogenicity avian influenza virus isolated from poultry in South Korea, 2022–2023. Virus Research. https://doi.org/10.1016/j.virusres.2025.199541</x:v>
+[7] Cha Ra Mi et al. (2025). Genetic characteristics and pathogenesis of clade 2.3.4.4b H5N1 high pathogenicity avian influenza virus isolated from poultry in South Korea, 2022–2023. Virus Research. https://doi.org/10.1016/j.virusres.2025.199541
+[8] Esaki Mana et al. (2025). Highly Pathogenic Avian Influenza A(H5N1) Outbreak in Endangered Cranes, Izumi Plain, Japan, 2022–23. Emerging Infectious Diseases. https://doi.org/10.3201/eid3105.241410</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="117" customHeight="1">
@@ -665,19 +711,22 @@
 [3] Cha Ra Mi et al. (2025). Genetic characteristics and pathogenesis of clade 2.3.4.4b H5N1 high pathogenicity avian influenza virus isolated from poultry in South Korea, 2022–2023. Virus Research. https://doi.org/10.1016/j.virusres.2025.199541</x:v>
       </x:c>
     </x:row>
-    <x:row r="17" ht="162" customHeight="1">
+    <x:row r="17" ht="207" customHeight="1">
       <x:c r="A17" s="7" t="str">
         <x:v>AS-c.2.1.1.1</x:v>
       </x:c>
       <x:c r="B17" s="7" t="str">
         <x:v>G2c-11 [1]
 Kor22-23C [2]
-22G8 [3]</x:v>
+22G8 [3]
+H5N1-I [4]
+H5N1-VII [4]</x:v>
       </x:c>
       <x:c r="C17" s="7" t="str">
         <x:v>[1] Takadate Yoshihiro et al. (2024). Genetic diversity of H5N1 and H5N2 high pathogenicity avian influenza viruses isolated from poultry in Japan during the winter of 2022–2023. Virus Research. https://doi.org/10.1016/j.virusres.2024.199425
 [2] Seo Ye-Ram et al. (2024). Evolution and Spread of Highly Pathogenic Avian Influenza A(H5N1) Clade 2.3.4.4b Virus in Wild Birds, South Korea, 2022–2023. Emerging Infectious Diseases. https://doi.org/10.3201/eid3002.231274
-[3] Cha Ra Mi et al. (2025). Genetic characteristics and pathogenesis of clade 2.3.4.4b H5N1 high pathogenicity avian influenza virus isolated from poultry in South Korea, 2022–2023. Virus Research. https://doi.org/10.1016/j.virusres.2025.199541</x:v>
+[3] Cha Ra Mi et al. (2025). Genetic characteristics and pathogenesis of clade 2.3.4.4b H5N1 high pathogenicity avian influenza virus isolated from poultry in South Korea, 2022–2023. Virus Research. https://doi.org/10.1016/j.virusres.2025.199541
+[4] Esaki Mana et al. (2025). Highly Pathogenic Avian Influenza A(H5N1) Outbreak in Endangered Cranes, Izumi Plain, Japan, 2022–23. Emerging Infectious Diseases. https://doi.org/10.3201/eid3105.241410</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="117" customHeight="1">
@@ -693,15 +742,17 @@
 [2] Cha Ra Mi et al. (2025). Genetic characteristics and pathogenesis of clade 2.3.4.4b H5N1 high pathogenicity avian influenza virus isolated from poultry in South Korea, 2022–2023. Virus Research. https://doi.org/10.1016/j.virusres.2025.199541</x:v>
       </x:c>
     </x:row>
-    <x:row r="19" ht="57" customHeight="1">
+    <x:row r="19" ht="102" customHeight="1">
       <x:c r="A19" s="6" t="str">
         <x:v>AS-c.2.1.1.3</x:v>
       </x:c>
       <x:c r="B19" s="6" t="str">
-        <x:v>G2c-4 [1]</x:v>
+        <x:v>G2c-4 [1]
+H5N1-II [2]</x:v>
       </x:c>
       <x:c r="C19" s="6" t="str">
-        <x:v>[1] Takadate Yoshihiro et al. (2024). Genetic diversity of H5N1 and H5N2 high pathogenicity avian influenza viruses isolated from poultry in Japan during the winter of 2022–2023. Virus Research. https://doi.org/10.1016/j.virusres.2024.199425</x:v>
+        <x:v>[1] Takadate Yoshihiro et al. (2024). Genetic diversity of H5N1 and H5N2 high pathogenicity avian influenza viruses isolated from poultry in Japan during the winter of 2022–2023. Virus Research. https://doi.org/10.1016/j.virusres.2024.199425
+[2] Esaki Mana et al. (2025). Highly Pathogenic Avian Influenza A(H5N1) Outbreak in Endangered Cranes, Izumi Plain, Japan, 2022–23. Emerging Infectious Diseases. https://doi.org/10.3201/eid3105.241410</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="102" customHeight="1">
@@ -789,12 +840,12 @@
 [2] Cha Ra Mi et al. (2026). Emergence and Genetic Characteristics of H5N1, H5N6, and H5N3 Clade 2.3.4.4b High Pathogenicity Avian Influenza Viruses in South Korea During the 2023–2024 and 2024–2025 Winter Seasons. Transboundary and Emerging Diseases. https://doi.org/10.1155/tbed/8053623</x:v>
       </x:c>
     </x:row>
-    <x:row r="27" ht="297" customHeight="1">
+    <x:row r="27" ht="342" customHeight="1">
       <x:c r="A27" s="7" t="str">
         <x:v>AS-d.1</x:v>
       </x:c>
       <x:c r="B27" s="7" t="str">
-        <x:v>G2d-0 [1]
+        <x:v>G2d-0 [1, 6]
 I [2]
 G1 [3]
 22G0 [4]
@@ -805,7 +856,8 @@
 [2] Hew Lim Yik et al. (2024). Continuous Introduction of H5 High Pathogenicity Avian Influenza Viruses in Hokkaido, Japan: Characterization of Viruses Isolated in Winter 2022–2023 and Early Winter 2023–2024. Transboundary and Emerging Diseases. https://doi.org/10.1155/2024/1199876
 [3] Cui Pengfei et al. (2022). Global dissemination of H5N1 influenza viruses bearing the clade 2.3.4.4b HA gene and biologic analysis of the ones detected in China. Emerging Microbes &amp; Infections. https://doi.org/10.1080/22221751.2022.2088407
 [4] Cha Ra Mi et al. (2025). Genetic characteristics and pathogenesis of clade 2.3.4.4b H5N1 high pathogenicity avian influenza virus isolated from poultry in South Korea, 2022–2023. Virus Research. https://doi.org/10.1016/j.virusres.2025.199541
-[5] Seo Ye-Ram et al. (2026). Multiple introductions and spread of novel reassortant highly pathogenic avian influenza A (H5N1) clade 2.3.4.4b viruses via wild birds, South Korea, 2024–2025. Veterinary Research, 57, 178. https://doi.org/10.1186/s13567-026-01847-2</x:v>
+[5] Seo Ye-Ram et al. (2026). Multiple introductions and spread of novel reassortant highly pathogenic avian influenza A (H5N1) clade 2.3.4.4b viruses via wild birds, South Korea, 2024–2025. Veterinary Research, 57, 178. https://doi.org/10.1186/s13567-026-01847-2
+[6] Takadate Yoshihiro et al. (2026). High pathogenicity avian influenza A (H5N1) viruses isolated from poultry and wild birds in Japan during the 2024–2025 season. Microbiology Spectrum. https://doi.org/10.1128/spectrum.00293-26</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="117" customHeight="1">
@@ -1642,4 +1694,161 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="26" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="29" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="55" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="19" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="23" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="23" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="55" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="100" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="55" customHeight="1">
+      <x:c r="A1" s="11" t="str">
+        <x:v>충돌 accession 검토</x:v>
+      </x:c>
+      <x:c r="B1" s="11" t="str"/>
+      <x:c r="C1" s="11" t="str"/>
+      <x:c r="D1" s="11" t="str"/>
+      <x:c r="E1" s="11" t="str"/>
+      <x:c r="F1" s="11" t="str"/>
+      <x:c r="G1" s="11" t="str"/>
+      <x:c r="H1" s="11" t="str"/>
+    </x:row>
+    <x:row r="2" ht="55" customHeight="1">
+      <x:c r="A2" s="11" t="str">
+        <x:v>아래 accession은 확정된 명칭 대응 근거 및 건수에서 제외. 원자료 genotype은 변경하지 않음.</x:v>
+      </x:c>
+      <x:c r="B2" s="11" t="str"/>
+      <x:c r="C2" s="11" t="str"/>
+      <x:c r="D2" s="11" t="str"/>
+      <x:c r="E2" s="11" t="str"/>
+      <x:c r="F2" s="11" t="str"/>
+      <x:c r="G2" s="11" t="str"/>
+      <x:c r="H2" s="11" t="str"/>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="11" t="str"/>
+      <x:c r="B3" s="11" t="str"/>
+      <x:c r="C3" s="11" t="str"/>
+      <x:c r="D3" s="11" t="str"/>
+      <x:c r="E3" s="11" t="str"/>
+      <x:c r="F3" s="11" t="str"/>
+      <x:c r="G3" s="11" t="str"/>
+      <x:c r="H3" s="11" t="str"/>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="13" t="str">
+        <x:v>Accession</x:v>
+      </x:c>
+      <x:c r="B4" s="13" t="str">
+        <x:v>출처</x:v>
+      </x:c>
+      <x:c r="C4" s="13" t="str">
+        <x:v>Strain</x:v>
+      </x:c>
+      <x:c r="D4" s="13" t="str">
+        <x:v>Collection date</x:v>
+      </x:c>
+      <x:c r="E4" s="13" t="str">
+        <x:v>Reported genotype</x:v>
+      </x:c>
+      <x:c r="F4" s="13" t="str">
+        <x:v>Current genotype</x:v>
+      </x:c>
+      <x:c r="G4" s="13" t="str">
+        <x:v>처리</x:v>
+      </x:c>
+      <x:c r="H4" s="13" t="str">
+        <x:v>Reference</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="100" customHeight="1">
+      <x:c r="A5" s="14" t="str">
+        <x:v>EPI_ISL_19645341</x:v>
+      </x:c>
+      <x:c r="B5" s="14" t="str">
+        <x:v>Table S2, No. 30</x:v>
+      </x:c>
+      <x:c r="C5" s="14" t="str">
+        <x:v>A/Eurasian_wigeon/Kagoshima/KU-24-4/2024</x:v>
+      </x:c>
+      <x:c r="D5" s="14" t="str">
+        <x:v>2024-11-18</x:v>
+      </x:c>
+      <x:c r="E5" s="14" t="str">
+        <x:v>G2d-0</x:v>
+      </x:c>
+      <x:c r="F5" s="14" t="str">
+        <x:v>AS-d.1</x:v>
+      </x:c>
+      <x:c r="G5" s="14" t="str">
+        <x:v>보류: 동일 논문 내 genotype 및 날짜 충돌</x:v>
+      </x:c>
+      <x:c r="H5" s="14" t="str">
+        <x:v>Takadate Yoshihiro et al. (2026). High pathogenicity avian influenza A (H5N1) viruses isolated from poultry and wild birds in Japan during the 2024–2025 season. Microbiology Spectrum. https://doi.org/10.1128/spectrum.00293-26</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="100" customHeight="1">
+      <x:c r="A6" s="14" t="str">
+        <x:v>EPI_ISL_19645341</x:v>
+      </x:c>
+      <x:c r="B6" s="14" t="str">
+        <x:v>Table S2, No. 105</x:v>
+      </x:c>
+      <x:c r="C6" s="14" t="str">
+        <x:v>A/Eurasian_wigeon/Kagoshima/KU-24-4/2024</x:v>
+      </x:c>
+      <x:c r="D6" s="14" t="str">
+        <x:v>2025-01-18</x:v>
+      </x:c>
+      <x:c r="E6" s="14" t="str">
+        <x:v>G2c-17</x:v>
+      </x:c>
+      <x:c r="F6" s="14" t="str">
+        <x:v>AS-d.1</x:v>
+      </x:c>
+      <x:c r="G6" s="14" t="str">
+        <x:v>보류: 확정 근거에서 제외</x:v>
+      </x:c>
+      <x:c r="H6" s="14" t="str">
+        <x:v>Takadate Yoshihiro et al. (2026). High pathogenicity avian influenza A (H5N1) viruses isolated from poultry and wild birds in Japan during the 2024–2025 season. Microbiology Spectrum. https://doi.org/10.1128/spectrum.00293-26</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="100" customHeight="1">
+      <x:c r="A7" s="14" t="str">
+        <x:v>EPI_ISL_19645341</x:v>
+      </x:c>
+      <x:c r="B7" s="14" t="str">
+        <x:v>현재 1705 isolates 데이터</x:v>
+      </x:c>
+      <x:c r="C7" s="14" t="str">
+        <x:v>A/Eurasian_wigeon/Kagoshima/KU-24-4/2023__(H5N1)</x:v>
+      </x:c>
+      <x:c r="D7" s="14" t="str">
+        <x:v>2024-11-18</x:v>
+      </x:c>
+      <x:c r="E7" s="14" t="str">
+        <x:v>HA_G2d</x:v>
+      </x:c>
+      <x:c r="F7" s="14" t="str">
+        <x:v>AS-d.1</x:v>
+      </x:c>
+      <x:c r="G7" s="14" t="str">
+        <x:v>분리주명 연도도 원문과 불일치. 원자료 유지.</x:v>
+      </x:c>
+      <x:c r="H7" s="14" t="str">
+        <x:v>fasttree_RAxML_중복1개제거_1705isolates_20261016.xlsx; 순서; no 529</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
 </file>
</xml_diff>

<commit_message>
Add seasonal 23G0 and 24G0 designations for AS-d.1
</commit_message>
<xml_diff>
--- a/docs/data/genotype_comparison_20261027.xlsx
+++ b/docs/data/genotype_comparison_20261027.xlsx
@@ -2,8 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="Ref5a0dba797f483e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Excluded accession" sheetId="2" r:id="Rfdd1f21d89ca4652"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="R6a370aeda1b64f04"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Excluded accession" sheetId="2" r:id="Ra48ebd708f434aec"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="명칭 연결 검토" sheetId="3" r:id="R6b8d8b28f3874a2d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -57,7 +58,7 @@
       <x:scheme val="minor"/>
     </x:font>
   </x:fonts>
-  <x:fills count="7">
+  <x:fills count="8">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -87,6 +88,11 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FFFFF2CC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFDCE7EF"/>
       </x:patternFill>
     </x:fill>
   </x:fills>
@@ -124,7 +130,7 @@
       <x:alignment vertical="center"/>
     </x:xf>
   </x:cellStyleXfs>
-  <x:cellXfs count="15">
+  <x:cellXfs count="17">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <x:alignment vertical="center"/>
     </x:xf>
@@ -168,6 +174,12 @@
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="4" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -840,7 +852,7 @@
 [2] Cha Ra Mi et al. (2026). Emergence and Genetic Characteristics of H5N1, H5N6, and H5N3 Clade 2.3.4.4b High Pathogenicity Avian Influenza Viruses in South Korea During the 2023–2024 and 2024–2025 Winter Seasons. Transboundary and Emerging Diseases. https://doi.org/10.1155/tbed/8053623</x:v>
       </x:c>
     </x:row>
-    <x:row r="27" ht="342" customHeight="1">
+    <x:row r="27" ht="409" customHeight="1">
       <x:c r="A27" s="7" t="str">
         <x:v>AS-d.1</x:v>
       </x:c>
@@ -849,7 +861,9 @@
 I [2]
 G1 [3]
 22G0 [4]
-Kor24–25B [5]</x:v>
+Kor24–25B [5]
+23G0 [7]
+24G0 [7]</x:v>
       </x:c>
       <x:c r="C27" s="7" t="str">
         <x:v>[1] Takadate Yoshihiro et al. (2024). Genetic diversity of H5N1 and H5N2 high pathogenicity avian influenza viruses isolated from poultry in Japan during the winter of 2022–2023. Virus Research. https://doi.org/10.1016/j.virusres.2024.199425
@@ -857,7 +871,8 @@
 [3] Cui Pengfei et al. (2022). Global dissemination of H5N1 influenza viruses bearing the clade 2.3.4.4b HA gene and biologic analysis of the ones detected in China. Emerging Microbes &amp; Infections. https://doi.org/10.1080/22221751.2022.2088407
 [4] Cha Ra Mi et al. (2025). Genetic characteristics and pathogenesis of clade 2.3.4.4b H5N1 high pathogenicity avian influenza virus isolated from poultry in South Korea, 2022–2023. Virus Research. https://doi.org/10.1016/j.virusres.2025.199541
 [5] Seo Ye-Ram et al. (2026). Multiple introductions and spread of novel reassortant highly pathogenic avian influenza A (H5N1) clade 2.3.4.4b viruses via wild birds, South Korea, 2024–2025. Veterinary Research, 57, 178. https://doi.org/10.1186/s13567-026-01847-2
-[6] Takadate Yoshihiro et al. (2026). High pathogenicity avian influenza A (H5N1) viruses isolated from poultry and wild birds in Japan during the 2024–2025 season. Microbiology Spectrum. https://doi.org/10.1128/spectrum.00293-26</x:v>
+[6] Takadate Yoshihiro et al. (2026). High pathogenicity avian influenza A (H5N1) viruses isolated from poultry and wild birds in Japan during the 2024–2025 season. Microbiology Spectrum. https://doi.org/10.1128/spectrum.00293-26
+[7] Cha Ra Mi et al. (2026). Emergence and Genetic Characteristics of H5N1, H5N6, and H5N3 Clade 2.3.4.4b High Pathogenicity Avian Influenza Viruses in South Korea During the 2023–2024 and 2024–2025 Winter Seasons. Transboundary and Emerging Diseases, 2026, 8053623. https://doi.org/10.1155/tbed/8053623</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="117" customHeight="1">
@@ -1851,4 +1866,139 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="27" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="26" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="77" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="36" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="110" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" s="16" t="str">
+        <x:v>사례</x:v>
+      </x:c>
+      <x:c r="B1" s="16" t="str">
+        <x:v>GenoFLU-Asia</x:v>
+      </x:c>
+      <x:c r="C1" s="16" t="str">
+        <x:v>검토 결과</x:v>
+      </x:c>
+      <x:c r="D1" s="16" t="str">
+        <x:v>반영 여부</x:v>
+      </x:c>
+      <x:c r="E1" s="16" t="str">
+        <x:v>근거</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" ht="130" customHeight="1">
+      <x:c r="A2" s="11" t="str">
+        <x:v>22G0 / 23G0 / 24G0</x:v>
+      </x:c>
+      <x:c r="B2" s="11" t="str">
+        <x:v>AS-d.1</x:v>
+      </x:c>
+      <x:c r="C2" s="11" t="str">
+        <x:v>논문이 동일 genotype의 연속 시즌 검출과 명칭을 명시</x:v>
+      </x:c>
+      <x:c r="D2" s="11" t="str">
+        <x:v>23G0 및 24G0 추가</x:v>
+      </x:c>
+      <x:c r="E2" s="11" t="str">
+        <x:v>Cha Ra Mi et al. (2026). Emergence and Genetic Characteristics of H5N1, H5N6, and H5N3 Clade 2.3.4.4b High Pathogenicity Avian Influenza Viruses in South Korea During the 2023–2024 and 2024–2025 Winter Seasons. Transboundary and Emerging Diseases, 2026, 8053623. https://doi.org/10.1155/tbed/8053623</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" ht="130" customHeight="1">
+      <x:c r="A3" s="11" t="str">
+        <x:v>G04 / G7</x:v>
+      </x:c>
+      <x:c r="B3" s="11" t="str">
+        <x:v>AS-a.3(N6)</x:v>
+      </x:c>
+      <x:c r="C3" s="11" t="str">
+        <x:v>Yang et al. (2025)가 G04와 Gu et al. (2022)의 G7이 동일하다고 명시. 두 명칭은 기존 표에 이미 존재.</x:v>
+      </x:c>
+      <x:c r="D3" s="11" t="str">
+        <x:v>기존 대응 유지</x:v>
+      </x:c>
+      <x:c r="E3" s="11" t="str">
+        <x:v>Yang Kang et al. (2025). Genetic diversity of highly pathogenic avian influenza H5N6 and H5N8 viruses in poultry markets in Guangdong, China, 2020-2022. Journal of Virology. https://doi.org/10.1128/jvi.01145-24</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="130" customHeight="1">
+      <x:c r="A4" s="11" t="str">
+        <x:v>20A / 20E / 21E</x:v>
+      </x:c>
+      <x:c r="B4" s="11" t="str">
+        <x:v>해당 없음</x:v>
+      </x:c>
+      <x:c r="C4" s="11" t="str">
+        <x:v>각각 G2a / G2b / G2d의 이전 HA subgroup 명칭. 전체 8분절 genotype 명칭이 아님.</x:v>
+      </x:c>
+      <x:c r="D4" s="11" t="str">
+        <x:v>genotype 동의어에 추가하지 않음</x:v>
+      </x:c>
+      <x:c r="E4" s="11" t="str">
+        <x:v>Mine Junki et al. (2024). Genetics of H5N1 and H5N8 High-Pathogenicity Avian Influenza Viruses Isolated in Japan in Winter 2021–2022. Viruses, 16, 358. https://doi.org/10.3390/v16030358</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="130" customHeight="1">
+      <x:c r="A5" s="11" t="str">
+        <x:v>24G0 + N3</x:v>
+      </x:c>
+      <x:c r="B5" s="11" t="str">
+        <x:v>AS-d.1과 동일시하지 않음</x:v>
+      </x:c>
+      <x:c r="C5" s="11" t="str">
+        <x:v>NA가 N3인 재편성 바이러스로 H5N1 24G0와 구분</x:v>
+      </x:c>
+      <x:c r="D5" s="11" t="str">
+        <x:v>AS-d.1 대응에서 제외</x:v>
+      </x:c>
+      <x:c r="E5" s="11" t="str">
+        <x:v>Cha Ra Mi et al. (2026). Emergence and Genetic Characteristics of H5N1, H5N6, and H5N3 Clade 2.3.4.4b High Pathogenicity Avian Influenza Viruses in South Korea During the 2023–2024 and 2024–2025 Winter Seasons. Transboundary and Emerging Diseases, 2026, 8053623. https://doi.org/10.1155/tbed/8053623</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="130" customHeight="1">
+      <x:c r="A6" s="11" t="str">
+        <x:v>21G1–21G4 / I–IV</x:v>
+      </x:c>
+      <x:c r="B6" s="11" t="str">
+        <x:v>미확정</x:v>
+      </x:c>
+      <x:c r="C6" s="11" t="str">
+        <x:v>후속 문헌에서 2021–2022 시즌 APQA genotype을 21G1–21G4로 언급하지만 각 명칭을 동일 분리주 또는 전체 분절 구성으로 직접 연결하지 못함.</x:v>
+      </x:c>
+      <x:c r="D6" s="11" t="str">
+        <x:v>일대일 대응 추가 보류</x:v>
+      </x:c>
+      <x:c r="E6" s="11" t="str">
+        <x:v>Cha Ra Mi et al. (2023). Genetic Characterization and Pathogenesis of H5N1 High Pathogenicity Avian Influenza Virus Isolated in South Korea during 2021–2022. Viruses, 15, 1403. https://doi.org/10.3390/v15061403</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="130" customHeight="1">
+      <x:c r="A7" s="11" t="str">
+        <x:v>23G1 / 24G1</x:v>
+      </x:c>
+      <x:c r="B7" s="11" t="str">
+        <x:v>동일시하지 않음</x:v>
+      </x:c>
+      <x:c r="C7" s="11" t="str">
+        <x:v>연도 뒤 숫자가 같다는 이유만으로 동일 genotype으로 연결할 근거 없음. 본문의 22G0 연결만 확정.</x:v>
+      </x:c>
+      <x:c r="D7" s="11" t="str">
+        <x:v>자동 병합하지 않음</x:v>
+      </x:c>
+      <x:c r="E7" s="11" t="str">
+        <x:v>Cha Ra Mi et al. (2026). Emergence and Genetic Characteristics of H5N1, H5N6, and H5N3 Clade 2.3.4.4b High Pathogenicity Avian Influenza Viruses in South Korea During the 2023–2024 and 2024–2025 Winter Seasons. Transboundary and Emerging Diseases, 2026, 8053623. https://doi.org/10.1155/tbed/8053623</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
 </file>
</xml_diff>